<commit_message>
chore: publish hosted MVP verification and restore coverage
</commit_message>
<xml_diff>
--- a/docs/examples/fictional-billing-review.xlsx
+++ b/docs/examples/fictional-billing-review.xlsx
@@ -271,8 +271,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="ReviewhistoryData" displayName="ReviewhistoryData" ref="A1:H2" headerRowCount="1">
-  <autoFilter ref="A1:H2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="ReviewhistoryData" displayName="ReviewhistoryData" ref="A1:H4" headerRowCount="1">
+  <autoFilter ref="A1:H4"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Finding"/>
     <tableColumn id="2" name="Sequence"/>
@@ -641,7 +641,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>RUN-a1cd522155e544a8bb6428d1ed1bccb8</t>
+          <t>RUN-2f9d4a5741894c8192199779ee7505ab</t>
         </is>
       </c>
     </row>
@@ -653,7 +653,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T14:54:57+00:00</t>
+          <t>2026-10-24T03:49:10+00:00</t>
         </is>
       </c>
     </row>
@@ -999,7 +999,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>5b209bc22ffea5912c8e2599eea3897e399a964831ae63f6d3fb28b88d3fdfe4</t>
+          <t>297cd72a7f68fb8a1efbdd5e5fe8557f6b3c444607d051543e1879ec29286dc5</t>
         </is>
       </c>
     </row>
@@ -2076,7 +2076,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>RATE-OT</t>
+          <t>RATE-REG</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -2096,11 +2096,11 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>overtime</t>
+          <t>standard</t>
         </is>
       </c>
       <c r="F2" s="4" t="n">
-        <v>97.5</v>
+        <v>65</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -2115,17 +2115,17 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T14:54:56.465124+00:00</t>
+          <t>2026-10-24T03:36:47.213437+00:00</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>MVP-IMPORTER</t>
+          <t>DEMO-REVIEWER</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>MVP-APPROVER</t>
+          <t>DEMO-APPROVER</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
@@ -2137,7 +2137,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>RATE-REG</t>
+          <t>RATE-OT</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -2157,11 +2157,11 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>standard</t>
+          <t>overtime</t>
         </is>
       </c>
       <c r="F3" s="4" t="n">
-        <v>65</v>
+        <v>97.5</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -2176,17 +2176,17 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T14:54:56.465124+00:00</t>
+          <t>2026-10-24T03:36:47.213437+00:00</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>MVP-IMPORTER</t>
+          <t>DEMO-REVIEWER</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>MVP-APPROVER</t>
+          <t>DEMO-APPROVER</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
@@ -2237,17 +2237,17 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T14:54:56.465124+00:00</t>
+          <t>2026-10-24T03:36:47.213437+00:00</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>MVP-IMPORTER</t>
+          <t>DEMO-REVIEWER</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>MVP-APPROVER</t>
+          <t>DEMO-APPROVER</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
@@ -2359,7 +2359,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>FIL-c92b9930c4a9494cb34e9fe1285ac7b5</t>
+          <t>FIL-267ef790311848fab084a8085f7a4bfa</t>
         </is>
       </c>
     </row>
@@ -2394,7 +2394,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>FIL-c92b9930c4a9494cb34e9fe1285ac7b5</t>
+          <t>FIL-267ef790311848fab084a8085f7a4bfa</t>
         </is>
       </c>
     </row>
@@ -2429,7 +2429,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>FIL-c92b9930c4a9494cb34e9fe1285ac7b5</t>
+          <t>FIL-267ef790311848fab084a8085f7a4bfa</t>
         </is>
       </c>
     </row>
@@ -2464,7 +2464,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>FIL-cd658c6954d3470db6c050f43a828425</t>
+          <t>FIL-76ece27ef4294fddbd15e01a77ca7187</t>
         </is>
       </c>
     </row>
@@ -2499,7 +2499,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>FIL-cd658c6954d3470db6c050f43a828425</t>
+          <t>FIL-76ece27ef4294fddbd15e01a77ca7187</t>
         </is>
       </c>
     </row>
@@ -2534,7 +2534,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>FIL-cd658c6954d3470db6c050f43a828425</t>
+          <t>FIL-76ece27ef4294fddbd15e01a77ca7187</t>
         </is>
       </c>
     </row>
@@ -2569,7 +2569,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>FIL-cd658c6954d3470db6c050f43a828425</t>
+          <t>FIL-76ece27ef4294fddbd15e01a77ca7187</t>
         </is>
       </c>
     </row>
@@ -2604,7 +2604,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>FIL-cd658c6954d3470db6c050f43a828425</t>
+          <t>FIL-76ece27ef4294fddbd15e01a77ca7187</t>
         </is>
       </c>
     </row>
@@ -2639,7 +2639,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>FIL-cd658c6954d3470db6c050f43a828425</t>
+          <t>FIL-76ece27ef4294fddbd15e01a77ca7187</t>
         </is>
       </c>
     </row>
@@ -2674,7 +2674,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>FIL-cd658c6954d3470db6c050f43a828425</t>
+          <t>FIL-76ece27ef4294fddbd15e01a77ca7187</t>
         </is>
       </c>
     </row>
@@ -2709,7 +2709,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>FIL-cd658c6954d3470db6c050f43a828425</t>
+          <t>FIL-76ece27ef4294fddbd15e01a77ca7187</t>
         </is>
       </c>
     </row>
@@ -2744,7 +2744,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>FIL-0b794cd58ddd4ee886e83e5a95611570</t>
+          <t>FIL-3900cdef3d6c4b1ebcd2a96d80984898</t>
         </is>
       </c>
     </row>
@@ -2779,7 +2779,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>FIL-0b794cd58ddd4ee886e83e5a95611570</t>
+          <t>FIL-3900cdef3d6c4b1ebcd2a96d80984898</t>
         </is>
       </c>
     </row>
@@ -2814,7 +2814,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>FIL-0b794cd58ddd4ee886e83e5a95611570</t>
+          <t>FIL-3900cdef3d6c4b1ebcd2a96d80984898</t>
         </is>
       </c>
     </row>
@@ -2849,7 +2849,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>FIL-0b794cd58ddd4ee886e83e5a95611570</t>
+          <t>FIL-3900cdef3d6c4b1ebcd2a96d80984898</t>
         </is>
       </c>
     </row>
@@ -2884,7 +2884,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>FIL-0b794cd58ddd4ee886e83e5a95611570</t>
+          <t>FIL-3900cdef3d6c4b1ebcd2a96d80984898</t>
         </is>
       </c>
     </row>
@@ -2919,7 +2919,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>FIL-0b794cd58ddd4ee886e83e5a95611570</t>
+          <t>FIL-3900cdef3d6c4b1ebcd2a96d80984898</t>
         </is>
       </c>
     </row>
@@ -2954,7 +2954,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>FIL-0b794cd58ddd4ee886e83e5a95611570</t>
+          <t>FIL-3900cdef3d6c4b1ebcd2a96d80984898</t>
         </is>
       </c>
     </row>
@@ -2989,7 +2989,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>FIL-0b794cd58ddd4ee886e83e5a95611570</t>
+          <t>FIL-3900cdef3d6c4b1ebcd2a96d80984898</t>
         </is>
       </c>
     </row>
@@ -3016,7 +3016,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3087,12 +3087,12 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>MVP-IMPORTER</t>
+          <t>DEMO-REVIEWER</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T14:54:57.809304+00:00</t>
+          <t>2026-10-24T03:42:12.800750+00:00</t>
         </is>
       </c>
       <c r="F2" s="2" t="n"/>
@@ -3103,7 +3103,79 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>1d026b346fd9e531ecd59a407aeaefb0af80c3bfeb28b6e58784b86eb8d5a733</t>
+          <t>05863e97bff9688be26d0fae27d91abba24e675ed4bd67a97dc19a9467f8e866</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>FND-001</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>reopen</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>DEMO-REVIEWER</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24T03:49:05.565441+00:00</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>(notes omitted)</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>05863e97bff9688be26d0fae27d91abba24e675ed4bd67a97dc19a9467f8e866</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>FND-001</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>confirm</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>DEMO-REVIEWER</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24T03:49:06.449505+00:00</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>(notes omitted)</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>05863e97bff9688be26d0fae27d91abba24e675ed4bd67a97dc19a9467f8e866</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Complete recurring billing review and invite-only team access
</commit_message>
<xml_diff>
--- a/docs/examples/fictional-billing-review.xlsx
+++ b/docs/examples/fictional-billing-review.xlsx
@@ -15,6 +15,7 @@
     <sheet name="Source lineage" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Review history" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Coverage gaps" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Follow-up" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Overview'!$1:$1</definedName>
@@ -25,6 +26,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Source lineage'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Review history'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'Coverage gaps'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="8">'Follow-up'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -296,6 +298,24 @@
     <tableColumn id="3" name="Coverage"/>
     <tableColumn id="4" name="Reason"/>
     <tableColumn id="5" name="Financial estimate"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="FollowupData" displayName="FollowupData" ref="A1:I4" headerRowCount="1">
+  <autoFilter ref="A1:I4"/>
+  <tableColumns count="9">
+    <tableColumn id="1" name="Case reference"/>
+    <tableColumn id="2" name="Facility"/>
+    <tableColumn id="3" name="Review basis"/>
+    <tableColumn id="4" name="Latest status"/>
+    <tableColumn id="5" name="Owner"/>
+    <tableColumn id="6" name="Correction / evidence reference"/>
+    <tableColumn id="7" name="Verified run"/>
+    <tableColumn id="8" name="Last evidence run"/>
+    <tableColumn id="9" name="Updated at"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -641,7 +661,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>RUN-2f9d4a5741894c8192199779ee7505ab</t>
+          <t>RUN-8b253c009f20445b859e8ae1e4cd0c1a</t>
         </is>
       </c>
     </row>
@@ -653,7 +673,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T03:49:10+00:00</t>
+          <t>2026-10-24T15:21:46+00:00</t>
         </is>
       </c>
     </row>
@@ -713,7 +733,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Current completed run</t>
+          <t>Completed run - original source evidence</t>
         </is>
       </c>
     </row>
@@ -824,7 +844,7 @@
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -854,7 +874,7 @@
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -864,7 +884,7 @@
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -874,7 +894,7 @@
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -999,7 +1019,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>297cd72a7f68fb8a1efbdd5e5fe8557f6b3c444607d051543e1879ec29286dc5</t>
+          <t>3e6149efb556e2d09cc763d21b18eeed8d064fd0b787e07bffc82fb37ce48a31</t>
         </is>
       </c>
     </row>
@@ -1106,7 +1126,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Confirmed discrepancy</t>
+          <t>Needs review</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -2076,7 +2096,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>RATE-REG</t>
+          <t>RATE-OT</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -2096,11 +2116,11 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>standard</t>
+          <t>overtime</t>
         </is>
       </c>
       <c r="F2" s="4" t="n">
-        <v>65</v>
+        <v>97.5</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -2115,7 +2135,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T03:36:47.213437+00:00</t>
+          <t>2026-10-24T15:21:46.453145+00:00</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -2130,14 +2150,14 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>EX-TABLE-82892444c004d89786fe97ea</t>
+          <t>EX-TABLE-a53914a6e81d1c9d6a00fc08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>RATE-OT</t>
+          <t>RATE-REG</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -2157,11 +2177,11 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>overtime</t>
+          <t>standard</t>
         </is>
       </c>
       <c r="F3" s="4" t="n">
-        <v>97.5</v>
+        <v>65</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -2176,7 +2196,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T03:36:47.213437+00:00</t>
+          <t>2026-10-24T15:21:46.453145+00:00</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -2191,7 +2211,7 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>EX-TABLE-82892444c004d89786fe97ea</t>
+          <t>EX-TABLE-a53914a6e81d1c9d6a00fc08</t>
         </is>
       </c>
     </row>
@@ -2237,7 +2257,7 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T03:36:47.213437+00:00</t>
+          <t>2026-10-24T15:21:46.453145+00:00</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -2252,7 +2272,7 @@
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>EX-TABLE-82892444c004d89786fe97ea</t>
+          <t>EX-TABLE-a53914a6e81d1c9d6a00fc08</t>
         </is>
       </c>
     </row>
@@ -2341,25 +2361,25 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>rates.xlsx</t>
+          <t>rates.csv</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Contract rates</t>
+          <t>CSV</t>
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>e1dc1a535d29d7642c1dc74227fc693bea7ffc4db67b891b3adba57127111f21</t>
+          <t>3e8c7c3699f79f5fc7de92c5c332608fddd5246e88d51b5caf78700bb4cc63b9</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>FIL-267ef790311848fab084a8085f7a4bfa</t>
+          <t>FIL-c4ecaf597c1f44b0983a1eeae031aad5</t>
         </is>
       </c>
     </row>
@@ -2376,25 +2396,25 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>rates.xlsx</t>
+          <t>rates.csv</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Contract rates</t>
+          <t>CSV</t>
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>e1dc1a535d29d7642c1dc74227fc693bea7ffc4db67b891b3adba57127111f21</t>
+          <t>3e8c7c3699f79f5fc7de92c5c332608fddd5246e88d51b5caf78700bb4cc63b9</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>FIL-267ef790311848fab084a8085f7a4bfa</t>
+          <t>FIL-c4ecaf597c1f44b0983a1eeae031aad5</t>
         </is>
       </c>
     </row>
@@ -2411,25 +2431,25 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>rates.xlsx</t>
+          <t>rates.csv</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Contract rates</t>
+          <t>CSV</t>
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>e1dc1a535d29d7642c1dc74227fc693bea7ffc4db67b891b3adba57127111f21</t>
+          <t>3e8c7c3699f79f5fc7de92c5c332608fddd5246e88d51b5caf78700bb4cc63b9</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>FIL-267ef790311848fab084a8085f7a4bfa</t>
+          <t>FIL-c4ecaf597c1f44b0983a1eeae031aad5</t>
         </is>
       </c>
     </row>
@@ -2446,25 +2466,25 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>work.xlsx</t>
+          <t>work.csv</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Time export</t>
+          <t>CSV</t>
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>c9cf0fef3e7015c7a10e2b6f61458b707db9dcc20dafe1718ebd7595ce2d067c</t>
+          <t>60a80ad879f7149b9d0afc3b77cf599cbc4a6261e365ffbb301668a42478086b</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>FIL-76ece27ef4294fddbd15e01a77ca7187</t>
+          <t>FIL-16e824b98d294209af96bf040cfb6089</t>
         </is>
       </c>
     </row>
@@ -2481,25 +2501,25 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>work.xlsx</t>
+          <t>work.csv</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Time export</t>
+          <t>CSV</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>c9cf0fef3e7015c7a10e2b6f61458b707db9dcc20dafe1718ebd7595ce2d067c</t>
+          <t>60a80ad879f7149b9d0afc3b77cf599cbc4a6261e365ffbb301668a42478086b</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>FIL-76ece27ef4294fddbd15e01a77ca7187</t>
+          <t>FIL-16e824b98d294209af96bf040cfb6089</t>
         </is>
       </c>
     </row>
@@ -2516,25 +2536,25 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>work.xlsx</t>
+          <t>work.csv</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Time export</t>
+          <t>CSV</t>
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>c9cf0fef3e7015c7a10e2b6f61458b707db9dcc20dafe1718ebd7595ce2d067c</t>
+          <t>60a80ad879f7149b9d0afc3b77cf599cbc4a6261e365ffbb301668a42478086b</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>FIL-76ece27ef4294fddbd15e01a77ca7187</t>
+          <t>FIL-16e824b98d294209af96bf040cfb6089</t>
         </is>
       </c>
     </row>
@@ -2551,25 +2571,25 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>work.xlsx</t>
+          <t>work.csv</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Time export</t>
+          <t>CSV</t>
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>c9cf0fef3e7015c7a10e2b6f61458b707db9dcc20dafe1718ebd7595ce2d067c</t>
+          <t>60a80ad879f7149b9d0afc3b77cf599cbc4a6261e365ffbb301668a42478086b</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>FIL-76ece27ef4294fddbd15e01a77ca7187</t>
+          <t>FIL-16e824b98d294209af96bf040cfb6089</t>
         </is>
       </c>
     </row>
@@ -2586,25 +2606,25 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>work.xlsx</t>
+          <t>work.csv</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Time export</t>
+          <t>CSV</t>
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>c9cf0fef3e7015c7a10e2b6f61458b707db9dcc20dafe1718ebd7595ce2d067c</t>
+          <t>60a80ad879f7149b9d0afc3b77cf599cbc4a6261e365ffbb301668a42478086b</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>FIL-76ece27ef4294fddbd15e01a77ca7187</t>
+          <t>FIL-16e824b98d294209af96bf040cfb6089</t>
         </is>
       </c>
     </row>
@@ -2621,25 +2641,25 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>work.xlsx</t>
+          <t>work.csv</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Time export</t>
+          <t>CSV</t>
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>c9cf0fef3e7015c7a10e2b6f61458b707db9dcc20dafe1718ebd7595ce2d067c</t>
+          <t>60a80ad879f7149b9d0afc3b77cf599cbc4a6261e365ffbb301668a42478086b</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>FIL-76ece27ef4294fddbd15e01a77ca7187</t>
+          <t>FIL-16e824b98d294209af96bf040cfb6089</t>
         </is>
       </c>
     </row>
@@ -2656,25 +2676,25 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>work.xlsx</t>
+          <t>work.csv</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Time export</t>
+          <t>CSV</t>
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>c9cf0fef3e7015c7a10e2b6f61458b707db9dcc20dafe1718ebd7595ce2d067c</t>
+          <t>60a80ad879f7149b9d0afc3b77cf599cbc4a6261e365ffbb301668a42478086b</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>FIL-76ece27ef4294fddbd15e01a77ca7187</t>
+          <t>FIL-16e824b98d294209af96bf040cfb6089</t>
         </is>
       </c>
     </row>
@@ -2691,25 +2711,25 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>work.xlsx</t>
+          <t>work.csv</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Time export</t>
+          <t>CSV</t>
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>c9cf0fef3e7015c7a10e2b6f61458b707db9dcc20dafe1718ebd7595ce2d067c</t>
+          <t>60a80ad879f7149b9d0afc3b77cf599cbc4a6261e365ffbb301668a42478086b</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>FIL-76ece27ef4294fddbd15e01a77ca7187</t>
+          <t>FIL-16e824b98d294209af96bf040cfb6089</t>
         </is>
       </c>
     </row>
@@ -2726,25 +2746,25 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>invoices.xlsx</t>
+          <t>invoices.csv</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Hospital statement</t>
+          <t>CSV</t>
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>10f374fc0d13641188ba13bbd7c72521c78e168ead4967a30d2927bc96472297</t>
+          <t>319246c56565c5a09399f9363f14708a3cb094034cd3e88b6410fe1bafa23fc5</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>FIL-3900cdef3d6c4b1ebcd2a96d80984898</t>
+          <t>FIL-6b9d9cb1ab004419ad711baff5d56c3e</t>
         </is>
       </c>
     </row>
@@ -2761,25 +2781,25 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>invoices.xlsx</t>
+          <t>invoices.csv</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Hospital statement</t>
+          <t>CSV</t>
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>10f374fc0d13641188ba13bbd7c72521c78e168ead4967a30d2927bc96472297</t>
+          <t>319246c56565c5a09399f9363f14708a3cb094034cd3e88b6410fe1bafa23fc5</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>FIL-3900cdef3d6c4b1ebcd2a96d80984898</t>
+          <t>FIL-6b9d9cb1ab004419ad711baff5d56c3e</t>
         </is>
       </c>
     </row>
@@ -2796,25 +2816,25 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>invoices.xlsx</t>
+          <t>invoices.csv</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Hospital statement</t>
+          <t>CSV</t>
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>10f374fc0d13641188ba13bbd7c72521c78e168ead4967a30d2927bc96472297</t>
+          <t>319246c56565c5a09399f9363f14708a3cb094034cd3e88b6410fe1bafa23fc5</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>FIL-3900cdef3d6c4b1ebcd2a96d80984898</t>
+          <t>FIL-6b9d9cb1ab004419ad711baff5d56c3e</t>
         </is>
       </c>
     </row>
@@ -2831,25 +2851,25 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>invoices.xlsx</t>
+          <t>invoices.csv</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Hospital statement</t>
+          <t>CSV</t>
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>10f374fc0d13641188ba13bbd7c72521c78e168ead4967a30d2927bc96472297</t>
+          <t>319246c56565c5a09399f9363f14708a3cb094034cd3e88b6410fe1bafa23fc5</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>FIL-3900cdef3d6c4b1ebcd2a96d80984898</t>
+          <t>FIL-6b9d9cb1ab004419ad711baff5d56c3e</t>
         </is>
       </c>
     </row>
@@ -2866,25 +2886,25 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>invoices.xlsx</t>
+          <t>invoices.csv</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Hospital statement</t>
+          <t>CSV</t>
         </is>
       </c>
       <c r="E17" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>10f374fc0d13641188ba13bbd7c72521c78e168ead4967a30d2927bc96472297</t>
+          <t>319246c56565c5a09399f9363f14708a3cb094034cd3e88b6410fe1bafa23fc5</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>FIL-3900cdef3d6c4b1ebcd2a96d80984898</t>
+          <t>FIL-6b9d9cb1ab004419ad711baff5d56c3e</t>
         </is>
       </c>
     </row>
@@ -2901,25 +2921,25 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>invoices.xlsx</t>
+          <t>invoices.csv</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Hospital statement</t>
+          <t>CSV</t>
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>10f374fc0d13641188ba13bbd7c72521c78e168ead4967a30d2927bc96472297</t>
+          <t>319246c56565c5a09399f9363f14708a3cb094034cd3e88b6410fe1bafa23fc5</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>FIL-3900cdef3d6c4b1ebcd2a96d80984898</t>
+          <t>FIL-6b9d9cb1ab004419ad711baff5d56c3e</t>
         </is>
       </c>
     </row>
@@ -2936,25 +2956,25 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>invoices.xlsx</t>
+          <t>invoices.csv</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Hospital statement</t>
+          <t>CSV</t>
         </is>
       </c>
       <c r="E19" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>10f374fc0d13641188ba13bbd7c72521c78e168ead4967a30d2927bc96472297</t>
+          <t>319246c56565c5a09399f9363f14708a3cb094034cd3e88b6410fe1bafa23fc5</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>FIL-3900cdef3d6c4b1ebcd2a96d80984898</t>
+          <t>FIL-6b9d9cb1ab004419ad711baff5d56c3e</t>
         </is>
       </c>
     </row>
@@ -2971,25 +2991,25 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>invoices.xlsx</t>
+          <t>invoices.csv</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Hospital statement</t>
+          <t>CSV</t>
         </is>
       </c>
       <c r="E20" s="2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>10f374fc0d13641188ba13bbd7c72521c78e168ead4967a30d2927bc96472297</t>
+          <t>319246c56565c5a09399f9363f14708a3cb094034cd3e88b6410fe1bafa23fc5</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>FIL-3900cdef3d6c4b1ebcd2a96d80984898</t>
+          <t>FIL-6b9d9cb1ab004419ad711baff5d56c3e</t>
         </is>
       </c>
     </row>
@@ -3074,110 +3094,98 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>FND-001</t>
+          <t>CASE-22f84051-1dec-4c7f-8837-b3b679ff1641</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>1</v>
+        <v>3239</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>confirm</t>
+          <t>identified</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>DEMO-REVIEWER</t>
+          <t>SYSTEM</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T03:42:12.800750+00:00</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="n"/>
+          <t>2026-10-24T11:21:46.743831-04:00</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr"/>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>(notes omitted)</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>05863e97bff9688be26d0fae27d91abba24e675ed4bd67a97dc19a9467f8e866</t>
-        </is>
-      </c>
+      <c r="H2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>FND-001</t>
+          <t>CASE-5323f682-e961-4672-99c0-05c66c0f5a51</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>2</v>
+        <v>3240</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>reopen</t>
+          <t>identified</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>DEMO-REVIEWER</t>
+          <t>SYSTEM</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T03:49:05.565441+00:00</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="n"/>
+          <t>2026-10-24T11:21:46.743831-04:00</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr"/>
       <c r="G3" s="2" t="inlineStr">
         <is>
           <t>(notes omitted)</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>05863e97bff9688be26d0fae27d91abba24e675ed4bd67a97dc19a9467f8e866</t>
-        </is>
-      </c>
+      <c r="H3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>FND-001</t>
+          <t>CASE-c2747590-a01b-4115-9be5-c12144b9837a</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>3</v>
+        <v>3241</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>confirm</t>
+          <t>identified</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>DEMO-REVIEWER</t>
+          <t>SYSTEM</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T03:49:06.449505+00:00</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="n"/>
+          <t>2026-10-24T11:21:46.743831-04:00</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr"/>
       <c r="G4" s="2" t="inlineStr">
         <is>
           <t>(notes omitted)</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>05863e97bff9688be26d0fae27d91abba24e675ed4bd67a97dc19a9467f8e866</t>
-        </is>
-      </c>
+      <c r="H4" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3308,4 +3316,193 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:I4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Case reference</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Facility</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Review basis</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Latest status</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Correction / evidence reference</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Verified run</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Last evidence run</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Updated at</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>CASE-22f84051-1dec-4c7f-8837-b3b679ff1641</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>FAC-A</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Approved rate mismatch</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>RUN-8b253c009f20445b859e8ae1e4cd0c1a</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24T11:21:46.743831-04:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>CASE-5323f682-e961-4672-99c0-05c66c0f5a51</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>FAC-A</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Unsupported component</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>RUN-8b253c009f20445b859e8ae1e4cd0c1a</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24T11:21:46.743831-04:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>CASE-c2747590-a01b-4115-9be5-c12144b9837a</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>FAC-A</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Time approval pending</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>RUN-8b253c009f20445b859e8ae1e4cd0c1a</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24T11:21:46.743831-04:00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;CShiftClarity | Fictional evaluation only | Page &amp;P</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>